<commit_message>
fix: remove example row from EDM test spreadsheet
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/edm_teste_campinas.xlsx
+++ b/examples/edm_teste_campinas.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NFS-e Campinas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,11 +30,8 @@
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
-    <font>
-      <b val="1"/>
-    </font>
   </fonts>
-  <fills count="7">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -49,22 +45,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DEEAF1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="002E75B6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00595959"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EBF3FB"/>
       </patternFill>
     </fill>
   </fills>
@@ -80,22 +66,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -461,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB3"/>
+  <dimension ref="A1:AB2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -636,109 +617,16 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="4" t="n">
+    <row r="2">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>01/2026</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Serviços de consultoria em tecnologia da informação</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>1.07</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="n">
-        <v>3500</v>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>Empresa Tomadora Ltda</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>12.345.678/0001-90</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr"/>
-      <c r="I2" s="4" t="inlineStr"/>
-      <c r="J2" s="4" t="inlineStr"/>
-      <c r="K2" s="4" t="inlineStr">
-        <is>
-          <t>financeiro@empresa.com.br</t>
-        </is>
-      </c>
-      <c r="L2" s="4" t="inlineStr">
-        <is>
-          <t>Rua Exemplo</t>
-        </is>
-      </c>
-      <c r="M2" s="4" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="N2" s="4" t="inlineStr">
-        <is>
-          <t>Sala 5</t>
-        </is>
-      </c>
-      <c r="O2" s="4" t="inlineStr">
-        <is>
-          <t>Centro</t>
-        </is>
-      </c>
-      <c r="P2" s="4" t="inlineStr">
-        <is>
-          <t>13010100</t>
-        </is>
-      </c>
-      <c r="Q2" s="4" t="inlineStr">
-        <is>
-          <t>3509502</t>
-        </is>
-      </c>
-      <c r="R2" s="4" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="S2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T2" s="4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="U2" s="4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V2" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="W2" s="4" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>04/2026</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Honorários Contábeis - Prestacao de servico em contabilidade
 Honorários Contábeis - Prestacao de servicos de Departamento Pessoal
@@ -746,299 +634,82 @@
 Contrato N. 2025/00103 - Ref. Abr/2026 - Vencto. 15/05/2026</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>17.19</t>
         </is>
       </c>
-      <c r="E3" s="6" t="n">
+      <c r="E2" t="n">
         <v>450</v>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>EDM ASSESSORIA ADMINISTRATIVA E TECNOLOGICA EIRELI</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>18.298.204/0001-16</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr"/>
-      <c r="I3" s="6" t="inlineStr"/>
-      <c r="J3" s="6" t="inlineStr"/>
-      <c r="K3" s="6" t="inlineStr">
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
         <is>
           <t>ericmaubr@gmail.com</t>
         </is>
       </c>
-      <c r="L3" s="6" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>R SALDANHA DA GAMA</t>
         </is>
       </c>
-      <c r="M3" s="6" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>244</t>
         </is>
       </c>
-      <c r="N3" s="6" t="inlineStr"/>
-      <c r="O3" s="6" t="inlineStr">
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
         <is>
           <t>LAPA</t>
         </is>
       </c>
-      <c r="P3" s="6" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>05081000</t>
         </is>
       </c>
-      <c r="Q3" s="6" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>3550308</t>
         </is>
       </c>
-      <c r="R3" s="6" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>SP</t>
         </is>
       </c>
-      <c r="S3" s="6" t="n">
+      <c r="S2" t="n">
         <v>0</v>
       </c>
-      <c r="T3" s="6" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="U3" s="6" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="V3" s="6" t="n">
+      <c r="V2" t="n">
         <v>1</v>
       </c>
-      <c r="W3" s="6" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>6920601</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A32"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="90" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>INSTRUÇÕES DE PREENCHIMENTO — NFS-e CAMPINAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>CAMPOS OBRIGATÓRIOS (marcados com *)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>numero_rps        Número sequencial do RPS. Cada linha deve ter um número único.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>competencia       Mês/ano de competência no formato MM/AAAA. Exemplo: 01/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>discriminacao     Descrição completa do serviço prestado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>codigo_servico    Código LC 116/2003. Exemplos: 1.07 (informática), 17.01 (assessoria).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>valor_servico     Valor dos serviços em reais. Use ponto como separador decimal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>tomador_razao_social  Nome ou razão social do tomador (cliente final).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>tomador_cnpj      CNPJ do tomador (pessoa jurídica). OU</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>tomador_cpf       CPF do tomador (pessoa física). Preencha um dos dois.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12"/>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>CAMPOS OPCIONAIS</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>data_emissao      Data de emissão no formato DD/MM/AAAA. Se vazio, usa a data de hoje.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>iss_retido        ISS retido na fonte? S ou N. Default: N</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>optante_simples   Tomador é optante pelo Simples Nacional? S ou N. Default: N</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>deducoes          Valor das deduções em reais. Default: 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>natureza_operacao 1=Tributação no município (default), 2=Fora do município</t>
-        </is>
-      </c>
-    </row>
-    <row r="19"/>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>RESULTADO (preenchido automaticamente após emissão)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>status            EMITIDA ou ERRO</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>numero_nfse       Número da NFS-e emitida.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>codigo_verificacao  Código de verificação para consulta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>link_consulta     URL para visualização/download da nota.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>erro              Mensagem de erro, se houver.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26"/>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>DICAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>- Mantenha a linha 1 (cabeçalho) sem alterações.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>- A linha 2 é apenas um exemplo; substitua pelos dados reais.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>- Adicione uma linha por nota fiscal a emitir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>- Código IBGE de Campinas: 3509502</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>- Códigos de serviço: consulte o ISS Campinas para o código municipal correto.</t>
         </is>
       </c>
     </row>

</xml_diff>